<commit_message>
added improved roi spreadsheet to submissions
</commit_message>
<xml_diff>
--- a/submissions/automation-opportunity-roi-model.xlsx
+++ b/submissions/automation-opportunity-roi-model.xlsx
@@ -41,15 +41,14 @@
         <t xml:space="preserve">Multiplier of 6 for numbers taken over 2 months.</t>
       </text>
     </comment>
-    <comment authorId="0" ref="J1">
+    <comment authorId="0" ref="I1">
       <text>
         <t xml:space="preserve">Can use ADKAR if stuck</t>
       </text>
     </comment>
-    <comment authorId="0" ref="C3">
+    <comment authorId="0" ref="C2">
       <text>
-        <t xml:space="preserve">These 2 can be achieved within the same low-complexity implementation, so value is effectively "halved".
-</t>
+        <t xml:space="preserve">Low-complexity implementation cost divided by number of opportunities that fall under "developing portal"</t>
       </text>
     </comment>
   </commentList>
@@ -57,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
   <si>
     <t>Assumption</t>
   </si>
@@ -305,6 +304,12 @@
     <t>Number of agents</t>
   </si>
   <si>
+    <t>Portal training cost</t>
+  </si>
+  <si>
+    <t>finance assumptions</t>
+  </si>
+  <si>
     <t>Opportunity</t>
   </si>
   <si>
@@ -317,21 +322,18 @@
     <t>Hours saved (Annual)</t>
   </si>
   <si>
-    <t>Cost saved</t>
-  </si>
-  <si>
     <t>Revenue uplift (Annually)</t>
   </si>
   <si>
-    <t>Net benefit</t>
-  </si>
-  <si>
     <t>Soft benefit</t>
   </si>
   <si>
     <t>12-month ROI</t>
   </si>
   <si>
+    <t>Payback Period (Years)</t>
+  </si>
+  <si>
     <t>Risks</t>
   </si>
   <si>
@@ -371,16 +373,7 @@
     <t>portal takes the responsibility of scheduling a follow up away from agent, by accessing and modifying all agents' schedules</t>
   </si>
   <si>
-    <t>waiting for gareth</t>
-  </si>
-  <si>
     <t>Less conflict, fairness to agents</t>
-  </si>
-  <si>
-    <t>Train agents</t>
-  </si>
-  <si>
-    <t>Train agents in how to navigate portal</t>
   </si>
 </sst>
 </file>
@@ -474,11 +467,11 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -626,7 +619,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E10" displayName="Table3" name="Table3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E11" displayName="Table3" name="Table3" id="3">
   <tableColumns count="5">
     <tableColumn name="Metric" id="1"/>
     <tableColumn name="Value" id="2"/>
@@ -639,20 +632,19 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L9" displayName="Table2" name="Table2" id="4">
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K8" displayName="Table2" name="Table2" id="4">
+  <tableColumns count="11">
     <tableColumn name="Opportunity" id="1"/>
     <tableColumn name="Description" id="2"/>
     <tableColumn name="Implementation Cost" id="3"/>
     <tableColumn name="Hours saved (Annual)" id="4"/>
-    <tableColumn name="Cost saved" id="5"/>
-    <tableColumn name="Revenue uplift (Annually)" id="6"/>
-    <tableColumn name="Net benefit" id="7"/>
-    <tableColumn name="Soft benefit" id="8"/>
-    <tableColumn name="12-month ROI" id="9"/>
-    <tableColumn name="Risks" id="10"/>
-    <tableColumn name="Confidence Level" id="11"/>
-    <tableColumn name="Priority" id="12"/>
+    <tableColumn name="Revenue uplift (Annually)" id="5"/>
+    <tableColumn name="Soft benefit" id="6"/>
+    <tableColumn name="12-month ROI" id="7"/>
+    <tableColumn name="Payback Period (Years)" id="8"/>
+    <tableColumn name="Risks" id="9"/>
+    <tableColumn name="Confidence Level" id="10"/>
+    <tableColumn name="Priority" id="11"/>
   </tableColumns>
   <tableStyleInfo name="Opportunities-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -1400,6 +1392,24 @@
         <v>69</v>
       </c>
     </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="7">
+        <f>20*B10*Assumptions!C7</f>
+        <v>25520</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">
@@ -1422,55 +1432,53 @@
     <col customWidth="1" min="5" max="5" width="13.75"/>
     <col customWidth="1" min="6" max="6" width="27.63"/>
     <col customWidth="1" min="7" max="7" width="13.75"/>
-    <col customWidth="1" min="8" max="9" width="14.25"/>
-    <col customWidth="1" min="10" max="10" width="15.63"/>
-    <col customWidth="1" min="11" max="11" width="18.38"/>
+    <col customWidth="1" min="8" max="8" width="21.38"/>
+    <col customWidth="1" min="9" max="10" width="14.25"/>
+    <col customWidth="1" min="11" max="11" width="15.63"/>
+    <col customWidth="1" min="12" max="12" width="18.38"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="H1" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>90</v>
       </c>
+      <c r="H1" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>92</v>
+      </c>
       <c r="J1" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="11">
         <f>(Assumptions!C16/4)</f>
@@ -1480,26 +1488,31 @@
         <f>ROUND(6347*6/(60),0)</f>
         <v>635</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="11">
+      <c r="E2" s="11">
         <f>D2*Assumptions!C7</f>
         <v>13970</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="I2" s="10"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
+      <c r="F2" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" s="12">
+        <f t="shared" ref="G2:G5" si="1">E2-C2</f>
+        <v>2720</v>
+      </c>
+      <c r="H2" s="13">
+        <f t="shared" ref="H2:H5" si="2">ROUND(C2/E2,1)</f>
+        <v>0.8</v>
+      </c>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C3" s="11">
         <f>(Assumptions!C16/4)</f>
@@ -1509,26 +1522,31 @@
         <f>ROUND(4285*6/(60),0)</f>
         <v>429</v>
       </c>
-      <c r="E3" s="12"/>
-      <c r="F3" s="11">
+      <c r="E3" s="11">
         <f>D3*Assumptions!C8</f>
         <v>9009</v>
       </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
+      <c r="F3" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="12">
+        <f t="shared" si="1"/>
+        <v>-2241</v>
+      </c>
+      <c r="H3" s="13">
+        <f t="shared" si="2"/>
+        <v>1.2</v>
+      </c>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" s="11">
         <f>Assumptions!C16/4</f>
@@ -1538,116 +1556,101 @@
         <f>ROUND(7580*6/(60),0)</f>
         <v>758</v>
       </c>
-      <c r="E4" s="12"/>
-      <c r="F4" s="11">
+      <c r="E4" s="11">
         <f>D4*Assumptions!C9</f>
         <v>288.04</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
+      <c r="F4" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" s="12">
+        <f t="shared" si="1"/>
+        <v>-10961.96</v>
+      </c>
+      <c r="H4" s="13">
+        <f t="shared" si="2"/>
+        <v>39.1</v>
+      </c>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" s="11">
         <f>Assumptions!C16/4</f>
         <v>11250</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="G5" s="12"/>
-      <c r="H5" s="10" t="s">
+      <c r="D5" s="10">
+        <f>ROUND(2*Metrics!B4*12/60,0)</f>
+        <v>1978</v>
+      </c>
+      <c r="E5" s="12">
+        <f>D5*Assumptions!C10</f>
+        <v>35604</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="I5" s="10"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
+      <c r="G5" s="12">
+        <f t="shared" si="1"/>
+        <v>24354</v>
+      </c>
+      <c r="H5" s="13">
+        <f t="shared" si="2"/>
+        <v>0.3</v>
+      </c>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" s="11">
-        <f>(20*Assumptions!C7)*Metrics!B10</f>
-        <v>25520</v>
-      </c>
-      <c r="D6" s="12" t="str">
-        <f>D2:D5</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C9 F2:F9">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C8 E2:E8">
       <formula1>AND(ISNUMBER(C2),(NOT(OR(NOT(ISERROR(DATEVALUE(C2))), AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>